<commit_message>
Edit DataCleaner to add nomr_volume option in the excel and metadata
</commit_message>
<xml_diff>
--- a/WP-2/Data_cleaning/ADNI_variables_cleaned1.xlsx
+++ b/WP-2/Data_cleaning/ADNI_variables_cleaned1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ifabfoundation-my.sharepoint.com/personal/chiara_pollicini_ifabfoundation_org/Documents/Documenti/Github/AIND/WP-2/Data_cleaning/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ifabfoundation-my.sharepoint.com/personal/raimondo_reggio_ifabfoundation_org/Documents/Desktop/GitHub/AIND/WP-2/Data_cleaning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_280D6BFD15627E0F62355476585DCE3A8746C57F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6257DB4-B8ED-4E18-94AD-28D79ADD1F02}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="11_280D6BFD15627E0F62355476585DCE3A8746C57F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{29D671AD-834F-4CFD-A18F-568193DBE471}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-2520" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1372" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1366" uniqueCount="294">
   <si>
     <t>file_name</t>
   </si>
@@ -899,13 +899,16 @@
   </si>
   <si>
     <t>0, 1, 2</t>
+  </si>
+  <si>
+    <t>volume</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -917,6 +920,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -954,11 +965,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -974,10 +986,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1533,9 +1541,6 @@
       <c r="L7" t="s">
         <v>21</v>
       </c>
-      <c r="M7" t="s">
-        <v>38</v>
-      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -1779,9 +1784,6 @@
       <c r="M13" t="s">
         <v>38</v>
       </c>
-      <c r="N13" t="s">
-        <v>65</v>
-      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -2190,7 +2192,7 @@
         <v>71</v>
       </c>
       <c r="N23" t="s">
-        <v>65</v>
+        <v>293</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
@@ -2231,7 +2233,7 @@
         <v>71</v>
       </c>
       <c r="N24" t="s">
-        <v>65</v>
+        <v>293</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
@@ -2272,7 +2274,7 @@
         <v>71</v>
       </c>
       <c r="N25" t="s">
-        <v>65</v>
+        <v>293</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
@@ -2313,7 +2315,7 @@
         <v>71</v>
       </c>
       <c r="N26" t="s">
-        <v>65</v>
+        <v>293</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
@@ -2354,7 +2356,7 @@
         <v>71</v>
       </c>
       <c r="N27" t="s">
-        <v>65</v>
+        <v>293</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
@@ -2391,11 +2393,8 @@
       <c r="L28" t="s">
         <v>21</v>
       </c>
-      <c r="M28" t="s">
-        <v>71</v>
-      </c>
       <c r="N28" t="s">
-        <v>65</v>
+        <v>293</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
@@ -2435,9 +2434,6 @@
       <c r="L29" t="s">
         <v>21</v>
       </c>
-      <c r="M29" t="s">
-        <v>71</v>
-      </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
@@ -2926,9 +2922,6 @@
       <c r="L42" t="s">
         <v>21</v>
       </c>
-      <c r="M42" t="s">
-        <v>71</v>
-      </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
@@ -3128,9 +3121,6 @@
       <c r="L47" t="s">
         <v>21</v>
       </c>
-      <c r="M47" t="s">
-        <v>38</v>
-      </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
@@ -5052,6 +5042,7 @@
       <c r="M124" t="s">
         <v>71</v>
       </c>
+      <c r="N124" s="2"/>
     </row>
     <row r="125" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
@@ -6395,5 +6386,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Risolto problema metadati (tranne volume_norm_value)
modifiche fatte:
- aggiunto pezzo a funzione update_new_support_file in managment_excel in modo che se re runno un file non devo cancellare il file o quelle righe ma viene ripristinato lo status di quel file nell'excel ==> vecchie variabili, così che si modifica assieme al DF man mano.
- in extraction metadata ho tolto le list comprehension che cercavano il parametro coincidente alla prefisso della variabile prima di '/' in quanto i metadati vengono salvati già nell'excel quando aggiungo le nuove variabilinel file di supporto e tolgo le precedenti. ==> risolto problema

Problema volume_norm_value identificato, il problema sono come sono chiamate nel jaison le variabili, prossima modificha che sarà implemetata
</commit_message>
<xml_diff>
--- a/WP-2/Data_cleaning/ADNI_variables_cleaned1.xlsx
+++ b/WP-2/Data_cleaning/ADNI_variables_cleaned1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ifabfoundation-my.sharepoint.com/personal/chiara_pollicini_ifabfoundation_org/Documents/Documenti/Github/AIND/WP-2/Data_cleaning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_3ECD1035D07F920E62355476585DCE3A8745D3C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61290D58-27C6-4CB7-A825-443AB2A988F1}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="11_3ECD1035D07F920E62355476585DCE3A8745D3C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCC6CE11-0305-4885-A456-E0425A495CF1}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-3705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2118" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2121" uniqueCount="367">
   <si>
     <t>file_name</t>
   </si>
@@ -1127,7 +1127,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1139,14 +1139,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1189,7 +1181,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1503,14 +1495,14 @@
     <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="55.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="34.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.21875" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="7.109375" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="7.88671875" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="4" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="4.88671875" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="3.6640625" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="3.21875" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="5.21875" hidden="1" customWidth="1"/>
     <col min="14" max="14" width="15.21875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="24.109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -1751,9 +1743,6 @@
       <c r="M6" t="s">
         <v>23</v>
       </c>
-      <c r="N6" t="s">
-        <v>38</v>
-      </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -1998,10 +1987,7 @@
         <v>23</v>
       </c>
       <c r="N12" t="s">
-        <v>65</v>
-      </c>
-      <c r="O12" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
@@ -2089,7 +2075,7 @@
         <v>65</v>
       </c>
       <c r="O14" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
@@ -2397,7 +2383,7 @@
         <v>65</v>
       </c>
       <c r="O21" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
@@ -2613,6 +2599,9 @@
       <c r="M26" t="s">
         <v>23</v>
       </c>
+      <c r="N26" t="s">
+        <v>65</v>
+      </c>
       <c r="O26" t="s">
         <v>91</v>
       </c>
@@ -2654,6 +2643,12 @@
       <c r="M27" t="s">
         <v>23</v>
       </c>
+      <c r="N27" t="s">
+        <v>65</v>
+      </c>
+      <c r="O27" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
@@ -3417,6 +3412,12 @@
       </c>
       <c r="M46" t="s">
         <v>23</v>
+      </c>
+      <c r="N46" t="s">
+        <v>65</v>
+      </c>
+      <c r="O46" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>